<commit_message>
Add repricer margin bounds and import history
</commit_message>
<xml_diff>
--- a/data/templates/portal-cost-template.xlsx
+++ b/data/templates/portal-cost-template.xlsx
@@ -8,6 +8,9 @@
     <sheet name="Справочник" sheetId="3" r:id="rId3"/>
     <sheet name="Ошибки_предыдущей_загрузки" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Заполнение'!A1:I1000</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -401,8 +404,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
+  <cols>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="44.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" t="str">
         <v>articleKey</v>
       </c>
@@ -431,7 +445,7 @@
         <v>reason</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="24" customHeight="1">
       <c r="A2" t="str">
         <v/>
       </c>
@@ -461,6 +475,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I1000"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
@@ -470,6 +485,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A3"/>
+  <cols>
+    <col min="1" max="1" width="115.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -496,6 +514,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -531,6 +553,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="72.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Add repricer MIN/MAX margin bounds and import history (#127)
Adds per-SKU MIN/MAX margin bounds, historical margin context, durable import-error history, updated Excel templates, and full validation tests.
</commit_message>
<xml_diff>
--- a/data/templates/portal-cost-template.xlsx
+++ b/data/templates/portal-cost-template.xlsx
@@ -8,6 +8,9 @@
     <sheet name="Справочник" sheetId="3" r:id="rId3"/>
     <sheet name="Ошибки_предыдущей_загрузки" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Заполнение'!A1:I1000</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -401,8 +404,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
+  <cols>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="44.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" t="str">
         <v>articleKey</v>
       </c>
@@ -431,7 +445,7 @@
         <v>reason</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="24" customHeight="1">
       <c r="A2" t="str">
         <v/>
       </c>
@@ -461,6 +475,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I1000"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
@@ -470,6 +485,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A3"/>
+  <cols>
+    <col min="1" max="1" width="115.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -496,6 +514,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -531,6 +553,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="72.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>